<commit_message>
Senj popravljeni instalacijski materijali i napravljeni markeri za terminale
</commit_message>
<xml_diff>
--- a/HE_Senj/materijal/instalacijski_materijal_Senj.xlsx
+++ b/HE_Senj/materijal/instalacijski_materijal_Senj.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\odojak\Brodotehna\Projekti\HE_Senj\materijal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC316736-9288-465A-8D62-8A119A19F926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C8E5E40-ACFA-4BD2-AF73-F0193461E73B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C49DCCE8-C980-47C6-9EFE-096C27DA3397}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="63">
   <si>
     <t>PRESJEK</t>
   </si>
@@ -74,24 +74,6 @@
     <t>TULJAK IZOL 2,5/8 PLAVI (100)</t>
   </si>
   <si>
-    <t>HA270803</t>
-  </si>
-  <si>
-    <t>TULJAK IZOL 0,75/8 SIVI (100)</t>
-  </si>
-  <si>
-    <t>HA270814</t>
-  </si>
-  <si>
-    <t>TULJAK IZOL 4/10 SIVI (100)</t>
-  </si>
-  <si>
-    <t>HA270818</t>
-  </si>
-  <si>
-    <t>TULJAK IZOL 6/12 ŽUTI (100)</t>
-  </si>
-  <si>
     <t>KOLIČINA</t>
   </si>
   <si>
@@ -104,30 +86,12 @@
     <t>N2XCH 2x10/10 mm²</t>
   </si>
   <si>
-    <t>STOPICA 16 mm²</t>
-  </si>
-  <si>
-    <t>STOPICA 10 mm²</t>
-  </si>
-  <si>
-    <t>STOPICA 2,5 mm²</t>
-  </si>
-  <si>
     <t>N2XCH 3x2,5/2,5 mm²</t>
   </si>
   <si>
     <t>N2XCH 2x2,5/2,5 mm²</t>
   </si>
   <si>
-    <t>KABEL</t>
-  </si>
-  <si>
-    <t>STOPICA 70 mm²</t>
-  </si>
-  <si>
-    <t>STOPICA 1,5 mm²</t>
-  </si>
-  <si>
     <t>HSLCH-JZ 12x1,5 mm²</t>
   </si>
   <si>
@@ -147,13 +111,130 @@
   </si>
   <si>
     <t>HSLCH-OZ 3x1,5 mm²</t>
+  </si>
+  <si>
+    <t>HA270805</t>
+  </si>
+  <si>
+    <t>TULJAK IZOL 1/8 CRVENI (500)</t>
+  </si>
+  <si>
+    <t>HA270822</t>
+  </si>
+  <si>
+    <t>TULJAK IZOL 10/12 CRVENI (100)</t>
+  </si>
+  <si>
+    <t>HA270826</t>
+  </si>
+  <si>
+    <t>TULJAK IZOL 16/12 PLAVI (100)</t>
+  </si>
+  <si>
+    <t>HA290988</t>
+  </si>
+  <si>
+    <t>STOPICA CIJEVNA 70/10 (25)</t>
+  </si>
+  <si>
+    <t>HA290952</t>
+  </si>
+  <si>
+    <t>STOPICA CIJEVNA 16/8 (100)</t>
+  </si>
+  <si>
+    <t>HA290942</t>
+  </si>
+  <si>
+    <t>STOPICA CIJEVNA 10/8 (100)</t>
+  </si>
+  <si>
+    <t>STOPICA CIJEVNA 2,5/5 (100)</t>
+  </si>
+  <si>
+    <t>HA290916</t>
+  </si>
+  <si>
+    <t>HA290908</t>
+  </si>
+  <si>
+    <t>STOPICA CIJEVNA 1,5/5 (100)</t>
+  </si>
+  <si>
+    <t>NAPOMENA</t>
+  </si>
+  <si>
+    <t>postoje pakiranja od 25 i 100 kom</t>
+  </si>
+  <si>
+    <t>postoje pakiranja od 25 i 500 kom</t>
+  </si>
+  <si>
+    <t>postoji pakiranje od 10 kom</t>
+  </si>
+  <si>
+    <t>moguća opcija HA290450</t>
+  </si>
+  <si>
+    <t>moguća opcija HA290412</t>
+  </si>
+  <si>
+    <t>moguća opcija HA290418 (50 kom)</t>
+  </si>
+  <si>
+    <t>DULJINA UKUPNO (m)</t>
+  </si>
+  <si>
+    <t>N2XCH 3x2.5/2.5 mm²</t>
+  </si>
+  <si>
+    <t>N2XCH 2x2.5/2.5 mm²</t>
+  </si>
+  <si>
+    <t>HSLCH 3x1.5 mm²</t>
+  </si>
+  <si>
+    <t>HSLCH-JZ 3x1.5 mm²</t>
+  </si>
+  <si>
+    <t>NYY-J 1x25 mm²</t>
+  </si>
+  <si>
+    <t>HSLCH-JZ 5x1.5 mm²</t>
+  </si>
+  <si>
+    <t>HSLCH-JZ 7x1.5 mm²</t>
+  </si>
+  <si>
+    <t>HSLCH 5x1.5 mm²</t>
+  </si>
+  <si>
+    <t>HSLCH-JZ 12x1.5 mm²</t>
+  </si>
+  <si>
+    <t>HSLCH 7x1.5 mm²</t>
+  </si>
+  <si>
+    <t>HSLCH-OZ 3x1.5 mm²</t>
+  </si>
+  <si>
+    <t>ETHERLINE Y CAT5 2X2XAWG22</t>
+  </si>
+  <si>
+    <t>OPTIKA</t>
+  </si>
+  <si>
+    <t>SHIRM KABELI</t>
+  </si>
+  <si>
+    <t>SVI KABELI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -176,22 +257,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -274,28 +355,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -304,6 +397,27 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="ColStyle7" xfId="1" xr:uid="{3EED7DA7-F8D0-4CC7-9509-DA0855E2A673}"/>
@@ -640,26 +754,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3214BBBB-04B2-4DEB-AB54-74889ECE6FF4}">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" customWidth="1"/>
     <col min="2" max="2" width="21.7109375" customWidth="1"/>
-    <col min="3" max="3" width="30.7109375" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" customWidth="1"/>
-    <col min="7" max="8" width="22.5703125" customWidth="1"/>
-    <col min="10" max="11" width="24.140625" customWidth="1"/>
+    <col min="3" max="4" width="30.7109375" customWidth="1"/>
+    <col min="5" max="5" width="34.28515625" style="17" customWidth="1"/>
+    <col min="6" max="7" width="11.85546875" customWidth="1"/>
+    <col min="8" max="9" width="22.5703125" customWidth="1"/>
+    <col min="11" max="12" width="24.140625" customWidth="1"/>
+    <col min="14" max="14" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="18"/>
+    </row>
+    <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>3</v>
       </c>
@@ -672,254 +790,448 @@
       <c r="D2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="E2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="12" t="s">
+      <c r="K2" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="L2" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="N2" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="O2" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="P2" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" s="11">
+        <v>120</v>
+      </c>
+      <c r="I3" s="12">
+        <f>4*2</f>
+        <v>8</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="L3" s="4">
+        <v>2</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="O3" s="20">
+        <v>2</v>
+      </c>
+      <c r="P3" s="4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4">
+        <f>2*I8</f>
+        <v>532</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4" s="11">
+        <v>25</v>
+      </c>
+      <c r="I4" s="12">
+        <v>1</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="4">
+        <v>2</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="O4" s="20">
+        <v>2</v>
+      </c>
+      <c r="P4" s="4">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5">
+        <f>2*I7</f>
+        <v>112</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" s="11">
+        <v>16</v>
+      </c>
+      <c r="I5" s="12">
+        <f>4*2</f>
+        <v>8</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="L5" s="4">
+        <v>2</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="O5" s="20">
+        <v>8</v>
+      </c>
+      <c r="P5" s="4">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
         <v>26</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6">
+        <f>2*I6</f>
+        <v>8</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" s="11">
+        <v>10</v>
+      </c>
+      <c r="I6" s="12">
+        <f>2*2</f>
+        <v>4</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="L6" s="4">
+        <v>8</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="O6" s="20">
+        <v>16</v>
+      </c>
+      <c r="P6" s="4">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7">
+        <f>2*I5</f>
+        <v>16</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="H7" s="6">
+        <v>2.5</v>
+      </c>
+      <c r="I7" s="3">
+        <f>3*8+2*16</f>
+        <v>56</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="L7" s="4">
+        <v>16</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="O7" s="20">
+        <v>4</v>
+      </c>
+      <c r="P7" s="4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H8" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="I8" s="15">
+        <f>3*4+3*22+5*5+7*4+5*1+12*9+7*1+3*5</f>
+        <v>266</v>
+      </c>
+      <c r="K8" s="7" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3">
-        <f>IFERROR(2*_xlfn.XLOOKUP(_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(C3,"IZOL "),"/")),$G$3:$G$8,$H$3:$H$8),"")</f>
-        <v>90</v>
-      </c>
-      <c r="G3" s="8">
-        <v>120</v>
-      </c>
-      <c r="H3" s="6">
-        <v>4</v>
-      </c>
-      <c r="J3" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="L8" s="4">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4">
-        <f>IFERROR(2*_xlfn.XLOOKUP(_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(C4,"IZOL "),"/")),$G$3:$G$8,$H$3:$H$8),"")</f>
-        <v>10</v>
-      </c>
-      <c r="G4" s="9">
-        <v>1.5</v>
-      </c>
-      <c r="H4" s="4">
-        <f>3+3+5+7+5+12+7+3</f>
-        <v>45</v>
-      </c>
-      <c r="J4" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" t="str">
-        <f>IFERROR(2*_xlfn.XLOOKUP(_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(C5,"IZOL "),"/")),$G$3:$G$8,$H$3:$H$8),"")</f>
-        <v/>
-      </c>
-      <c r="G5" s="8">
-        <v>16</v>
-      </c>
-      <c r="H5" s="6">
-        <v>4</v>
-      </c>
-      <c r="J5" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="K5" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" t="str">
-        <f>IFERROR(2*_xlfn.XLOOKUP(_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(C6,"IZOL "),"/")),$G$3:$G$8,$H$3:$H$8),"")</f>
-        <v/>
-      </c>
-      <c r="G6" s="9">
-        <v>2.5</v>
-      </c>
-      <c r="H6" s="3">
-        <f>3+2</f>
-        <v>5</v>
-      </c>
-      <c r="J6" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="K6" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" t="str">
-        <f>IFERROR(2*_xlfn.XLOOKUP(_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(C7,"IZOL "),"/")),$G$3:$G$8,$H$3:$H$8),"")</f>
-        <v/>
-      </c>
-      <c r="G7" s="8">
-        <v>25</v>
-      </c>
-      <c r="H7" s="6">
-        <v>1</v>
-      </c>
-      <c r="J7" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="K7" s="4">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G8" s="10">
-        <v>10</v>
-      </c>
-      <c r="H8" s="7">
-        <v>2</v>
-      </c>
-      <c r="J8" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="K8" s="4">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="N8" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="O8" s="20">
+        <v>22</v>
+      </c>
+      <c r="P8" s="4">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D9">
         <v>2</v>
       </c>
-      <c r="J9" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="K9" s="4">
+      <c r="E9" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="L9" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="N9" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="O9" s="20">
+        <v>1</v>
+      </c>
+      <c r="P9" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="D10">
         <v>2</v>
       </c>
-      <c r="J10" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="K10" s="4">
+      <c r="E10" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="L10" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="N10" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="O10" s="20">
+        <v>2</v>
+      </c>
+      <c r="P10" s="4">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
       <c r="C11" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
-      <c r="J11" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="K11" s="4">
+      <c r="E11" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="L11" s="4">
         <v>22</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="N11" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="O11" s="20">
+        <v>5</v>
+      </c>
+      <c r="P11" s="4">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>37</v>
+      </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="D12">
         <f>16+8</f>
         <v>24</v>
       </c>
-      <c r="J12" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="K12" s="4">
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="K12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L12" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="N12" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="O12" s="20">
+        <v>4</v>
+      </c>
+      <c r="P12" s="4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
       <c r="C13" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D13">
-        <f>SUM(K8:K14)</f>
+        <f>SUM(L8:L14)</f>
         <v>47</v>
       </c>
-      <c r="J13" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="K13" s="4">
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="K13" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L13" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="J14" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="K14" s="4">
+      <c r="N13" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="O13" s="20">
+        <v>1</v>
+      </c>
+      <c r="P13" s="4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="K14" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="L14" s="15">
         <v>5</v>
+      </c>
+      <c r="N14" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="O14" s="20">
+        <v>9</v>
+      </c>
+      <c r="P14" s="4">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N15" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="O15" s="20">
+        <v>1</v>
+      </c>
+      <c r="P15" s="4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N16" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="O16" s="20">
+        <v>5</v>
+      </c>
+      <c r="P16" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="14:16" x14ac:dyDescent="0.25">
+      <c r="N17" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="O17" s="20">
+        <v>3</v>
+      </c>
+      <c r="P17" s="4">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="18" spans="14:16" x14ac:dyDescent="0.25">
+      <c r="N18" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="O18" s="21">
+        <v>1</v>
+      </c>
+      <c r="P18" s="15">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Senj. Promjene u Y BJP12 ormaru. Dodani cable i terminal diagrami. Cut-outi uvodnica u GH001 i popravljene greske.
</commit_message>
<xml_diff>
--- a/HE_Senj/materijal/instalacijski_materijal_Senj.xlsx
+++ b/HE_Senj/materijal/instalacijski_materijal_Senj.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\odojak\Brodotehna\Projekti\HE_Senj\materijal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C8E5E40-ACFA-4BD2-AF73-F0193461E73B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EEB2489-9F42-48F2-AF3E-FEB9852B01EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C49DCCE8-C980-47C6-9EFE-096C27DA3397}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="64">
   <si>
     <t>PRESJEK</t>
   </si>
@@ -228,6 +228,9 @@
   </si>
   <si>
     <t>SVI KABELI</t>
+  </si>
+  <si>
+    <t>UKUPNO ŽILA (po tipu kabela)</t>
   </si>
 </sst>
 </file>
@@ -381,7 +384,7 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -394,13 +397,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -412,12 +408,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="ColStyle7" xfId="1" xr:uid="{3EED7DA7-F8D0-4CC7-9509-DA0855E2A673}"/>
@@ -754,30 +753,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3214BBBB-04B2-4DEB-AB54-74889ECE6FF4}">
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" customWidth="1"/>
     <col min="2" max="2" width="21.7109375" customWidth="1"/>
     <col min="3" max="4" width="30.7109375" customWidth="1"/>
-    <col min="5" max="5" width="34.28515625" style="17" customWidth="1"/>
+    <col min="5" max="5" width="34.28515625" style="14" customWidth="1"/>
     <col min="6" max="7" width="11.85546875" customWidth="1"/>
     <col min="8" max="9" width="22.5703125" customWidth="1"/>
     <col min="11" max="12" width="24.140625" customWidth="1"/>
     <col min="14" max="14" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="22" customWidth="1"/>
+    <col min="17" max="17" width="27.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
       <c r="E1" s="18"/>
     </row>
-    <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>3</v>
       </c>
@@ -808,27 +808,30 @@
       <c r="N2" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="O2" s="19" t="s">
+      <c r="O2" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="P2" s="15" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="Q2" s="9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>24</v>
       </c>
       <c r="C3" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="E3" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="H3" s="11">
+      <c r="H3" s="6">
         <v>120</v>
       </c>
-      <c r="I3" s="12">
+      <c r="I3" s="3">
         <f>4*2</f>
         <v>8</v>
       </c>
@@ -841,14 +844,18 @@
       <c r="N3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="O3" s="20">
+      <c r="O3" s="19">
         <v>2</v>
       </c>
-      <c r="P3" s="4">
+      <c r="P3" s="19">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q3" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N3," "),"x"))*O3</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>7</v>
       </c>
@@ -856,16 +863,16 @@
         <v>8</v>
       </c>
       <c r="D4">
-        <f>2*I8</f>
+        <f>2*SUMIF($N$3:$N$18,"*"&amp;SUBSTITUTE(_xlfn.TEXTAFTER(_xlfn.TEXTBEFORE(C4,"/"),"IZOL "),",",".")&amp;"*",$Q$3:$Q$18)</f>
         <v>532</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="6">
         <v>25</v>
       </c>
-      <c r="I4" s="12">
+      <c r="I4" s="3">
         <v>1</v>
       </c>
       <c r="K4" s="7" t="s">
@@ -877,14 +884,18 @@
       <c r="N4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O4" s="20">
+      <c r="O4" s="19">
         <v>2</v>
       </c>
-      <c r="P4" s="4">
+      <c r="P4" s="19">
         <v>200</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q4" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N4," "),"x"))*O4</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>9</v>
       </c>
@@ -892,16 +903,16 @@
         <v>10</v>
       </c>
       <c r="D5">
-        <f>2*I7</f>
+        <f t="shared" ref="D5:D7" si="0">2*SUMIF($N$3:$N$18,"*"&amp;SUBSTITUTE(_xlfn.TEXTAFTER(_xlfn.TEXTBEFORE(C5,"/"),"IZOL "),",",".")&amp;"*",$Q$3:$Q$18)</f>
         <v>112</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="6">
         <v>16</v>
       </c>
-      <c r="I5" s="12">
+      <c r="I5" s="3">
         <f>4*2</f>
         <v>8</v>
       </c>
@@ -914,14 +925,18 @@
       <c r="N5" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="O5" s="20">
+      <c r="O5" s="19">
         <v>8</v>
       </c>
-      <c r="P5" s="4">
+      <c r="P5" s="19">
         <v>405</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q5" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N5," "),"x"))*O5</f>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>26</v>
       </c>
@@ -929,16 +944,16 @@
         <v>27</v>
       </c>
       <c r="D6">
-        <f>2*I6</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="6">
         <v>10</v>
       </c>
-      <c r="I6" s="12">
+      <c r="I6" s="3">
         <f>2*2</f>
         <v>4</v>
       </c>
@@ -951,14 +966,18 @@
       <c r="N6" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="O6" s="20">
+      <c r="O6" s="19">
         <v>16</v>
       </c>
-      <c r="P6" s="4">
+      <c r="P6" s="19">
         <v>680</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q6" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N6," "),"x"))*O6</f>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>28</v>
       </c>
@@ -966,10 +985,10 @@
         <v>29</v>
       </c>
       <c r="D7">
-        <f>2*I5</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="14" t="s">
         <v>43</v>
       </c>
       <c r="H7" s="6">
@@ -988,18 +1007,22 @@
       <c r="N7" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="O7" s="20">
+      <c r="O7" s="19">
         <v>4</v>
       </c>
-      <c r="P7" s="4">
+      <c r="P7" s="19">
         <v>45</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="H8" s="14">
+      <c r="Q7" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N7," "),"x"))*O7</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="H8" s="11">
         <v>1.5</v>
       </c>
-      <c r="I8" s="15">
+      <c r="I8" s="12">
         <f>3*4+3*22+5*5+7*4+5*1+12*9+7*1+3*5</f>
         <v>266</v>
       </c>
@@ -1012,14 +1035,18 @@
       <c r="N8" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="O8" s="20">
+      <c r="O8" s="19">
         <v>22</v>
       </c>
-      <c r="P8" s="4">
+      <c r="P8" s="19">
         <v>475</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q8" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N8," "),"x"))*O8</f>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>30</v>
       </c>
@@ -1029,7 +1056,7 @@
       <c r="D9">
         <v>2</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="14" t="s">
         <v>44</v>
       </c>
       <c r="K9" s="7" t="s">
@@ -1041,14 +1068,18 @@
       <c r="N9" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="O9" s="20">
+      <c r="O9" s="19">
         <v>1</v>
       </c>
-      <c r="P9" s="4">
+      <c r="P9" s="19">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q9" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N9," "),"x"))*O9</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>32</v>
       </c>
@@ -1058,7 +1089,7 @@
       <c r="D10">
         <v>2</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="14" t="s">
         <v>46</v>
       </c>
       <c r="K10" s="7" t="s">
@@ -1070,14 +1101,18 @@
       <c r="N10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="O10" s="20">
+      <c r="O10" s="19">
         <v>2</v>
       </c>
-      <c r="P10" s="4">
+      <c r="P10" s="19">
         <v>299</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q10" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N10," "),"x"))*O10</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>34</v>
       </c>
@@ -1087,7 +1122,7 @@
       <c r="D11">
         <v>2</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="14" t="s">
         <v>45</v>
       </c>
       <c r="K11" s="7" t="s">
@@ -1099,14 +1134,18 @@
       <c r="N11" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="O11" s="20">
+      <c r="O11" s="19">
         <v>5</v>
       </c>
-      <c r="P11" s="4">
+      <c r="P11" s="19">
         <v>140</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q11" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N11," "),"x"))*O11</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>37</v>
       </c>
@@ -1117,8 +1156,8 @@
         <f>16+8</f>
         <v>24</v>
       </c>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
       <c r="K12" s="7" t="s">
         <v>21</v>
       </c>
@@ -1128,14 +1167,18 @@
       <c r="N12" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="O12" s="20">
+      <c r="O12" s="19">
         <v>4</v>
       </c>
-      <c r="P12" s="4">
+      <c r="P12" s="19">
         <v>90</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q12" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N12," "),"x"))*O12</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>38</v>
       </c>
@@ -1146,8 +1189,8 @@
         <f>SUM(L8:L14)</f>
         <v>47</v>
       </c>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
       <c r="K13" s="7" t="s">
         <v>22</v>
       </c>
@@ -1157,75 +1200,93 @@
       <c r="N13" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="O13" s="20">
+      <c r="O13" s="19">
         <v>1</v>
       </c>
-      <c r="P13" s="4">
+      <c r="P13" s="19">
         <v>65</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="K14" s="16" t="s">
+      <c r="Q13" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N13," "),"x"))*O13</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="K14" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="L14" s="15">
+      <c r="L14" s="12">
         <v>5</v>
       </c>
       <c r="N14" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="O14" s="20">
+      <c r="O14" s="19">
         <v>9</v>
       </c>
-      <c r="P14" s="4">
+      <c r="P14" s="19">
         <v>240</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q14" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N14," "),"x"))*O14</f>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="N15" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="O15" s="20">
+      <c r="O15" s="19">
         <v>1</v>
       </c>
-      <c r="P15" s="4">
+      <c r="P15" s="19">
         <v>65</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q15" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N15," "),"x"))*O15</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="N16" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="O16" s="20">
+      <c r="O16" s="19">
         <v>5</v>
       </c>
-      <c r="P16" s="4">
+      <c r="P16" s="19">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="14:16" x14ac:dyDescent="0.25">
+      <c r="Q16" s="4">
+        <f>_xlfn.NUMBERVALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(N16," "),"x"))*O16</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="14:17" x14ac:dyDescent="0.25">
       <c r="N17" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="O17" s="20">
+      <c r="O17" s="19">
         <v>3</v>
       </c>
-      <c r="P17" s="4">
+      <c r="P17" s="19">
         <v>120</v>
       </c>
-    </row>
-    <row r="18" spans="14:16" x14ac:dyDescent="0.25">
-      <c r="N18" s="16" t="s">
+      <c r="Q17" s="4"/>
+    </row>
+    <row r="18" spans="14:17" x14ac:dyDescent="0.25">
+      <c r="N18" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="O18" s="21">
+      <c r="O18" s="16">
         <v>1</v>
       </c>
-      <c r="P18" s="15">
+      <c r="P18" s="16">
         <v>90</v>
       </c>
+      <c r="Q18" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>